<commit_message>
docs(ai): 2027 AI budget sheet - Gemini 3.8 Flash for auto-replies
Owner, 2026-10-08: AI goes into next year's budget; Gemini 3.8 for the
auto-replies. New first sheet 'Budget 2027': adjustable inputs (measured
volume: ~1,000 chats/month, 6 customer messages per chat; measured helper
token sizes from the AI log), auto-reply and agent-helper lines, 20%
contingency, monthly and yearly totals in USD and SAR for Gemini 3.8 at
its 2027 price (the budget line), its 2026 price, GPT-5.6 Luna and the
current Gemini 2.5 Flash. Prices sheet gains both Gemini 3.8 rates.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ai/ai-cost-estimate.xlsx
+++ b/docs/ai/ai-cost-estimate.xlsx
@@ -4,13 +4,14 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimate" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick reply usage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget 2027" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimate" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick reply usage" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,11 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="#,##0&quot; SAR&quot;"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="#,##0&quot; SAR&quot;"/>
+    <numFmt numFmtId="167" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +63,10 @@
     <font>
       <name val="Arial"/>
       <color rgb="00008000"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -106,26 +113,49 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -498,25 +528,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI cost estimate - inputs</t>
+          <t>AI budget 2027 - Sara CRM</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Blue cells are inputs: change them and every total recalculates. Yellow = the levers you will most likely change.</t>
+          <t>Blue = inputs you can change. Measured = from the CRM itself (production, Sep-Oct 2026). Every total recalculates.</t>
         </is>
       </c>
     </row>
@@ -543,22 +575,23 @@
           <t>Chats per month (today)</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>1000</v>
+      <c r="B5" s="5">
+        <f>Inputs!B5</f>
+        <v/>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Production 28 Sep - 7 Oct 2026: 298 chats in ~9 days = about 1,000/month.</t>
+          <t>Measured: 344 chats in 10.5 days since go-live.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Growth multiplier</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
+          <t>Growth multiplier for 2027</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="n">
         <v>6</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -570,105 +603,474 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>AI calls per chat (agent helper)</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>5</v>
+          <t>Customer messages per chat</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="n">
+        <v>6</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Assumption: summaries, suggested replies, sentiment, enhance. Replace with the real figure from the ai_calls log after a few weeks.</t>
+          <t>Measured: 2,060 customer messages / 344 chats = 6.0.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Input tokens per helper call</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>1500</v>
+          <t>Share of customer messages answered by AI (auto-reply)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>0.5</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Assumption: system prompt + chat history. Avg chat = 11 messages / ~630 characters (production).</t>
+          <t>Planned automation of basic interactions. 0.5 = half; 1 = every message.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Output tokens per helper call</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>300</v>
+          <t>Input tokens per auto-reply</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>3000</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Assumption.</t>
+          <t>Instructions + the chat so far + order context, sent each time.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Customer messages per month (today)</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>5700</v>
+          <t>Output tokens per auto-reply</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>150</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Production: 1,717 customer messages in ~9 days = about 5,700/month.</t>
+          <t>A short chat reply.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Input tokens per automated reply</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>3000</v>
+          <t>Thinking tokens per auto-reply</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>400</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Assumption: full chat history + instructions + order context, sent on every customer message.</t>
+          <t>Gemini 3.8 thinks before answering and bills it as output. Set to ~100 with thinking on "low".</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Output tokens per automated reply</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>150</v>
+          <t>Agent-helper AI calls per chat</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="n">
+        <v>2</v>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Assumption: a short chat reply.</t>
+          <t>Summaries, suggested replies, enhance. Measured today: almost 0 (2 calls logged) - 2 assumes agents adopt it.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>Input tokens per helper call</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Measured from the AI log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Output tokens per helper call</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Measured from the AI log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Thinking tokens per helper call</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>390</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Measured from the AI log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Headroom for growth spikes, retries and price changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>USD to SAR</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="B17" s="13">
+        <f>Inputs!B13</f>
+        <v/>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Fixed peg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Per month (USD) unless stated</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Gemini 3.8 Flash - 2027 price (BUDGET)</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Gemini 3.8 Flash - 2026 price</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Luna</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Flash (current)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Customer messages per month</t>
+        </is>
+      </c>
+      <c r="B21" s="15">
+        <f>$B$5*$B$6*$B$7</f>
+        <v/>
+      </c>
+      <c r="C21" s="15">
+        <f>$B$5*$B$6*$B$7</f>
+        <v/>
+      </c>
+      <c r="D21" s="15">
+        <f>$B$5*$B$6*$B$7</f>
+        <v/>
+      </c>
+      <c r="E21" s="15">
+        <f>$B$5*$B$6*$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Auto-replies per month</t>
+        </is>
+      </c>
+      <c r="B22" s="15">
+        <f>$B$5*$B$6*$B$7*$B$8</f>
+        <v/>
+      </c>
+      <c r="C22" s="15">
+        <f>$B$5*$B$6*$B$7*$B$8</f>
+        <v/>
+      </c>
+      <c r="D22" s="15">
+        <f>$B$5*$B$6*$B$7*$B$8</f>
+        <v/>
+      </c>
+      <c r="E22" s="15">
+        <f>$B$5*$B$6*$B$7*$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Auto-replies cost</t>
+        </is>
+      </c>
+      <c r="B23" s="32">
+        <f>$B$5*$B$6*$B$7*$B$8*($B$9*Prices!D6+($B$10+$B$11)*Prices!E6)/1000000</f>
+        <v/>
+      </c>
+      <c r="C23" s="32">
+        <f>$B$5*$B$6*$B$7*$B$8*($B$9*Prices!D5+($B$10+$B$11)*Prices!E5)/1000000</f>
+        <v/>
+      </c>
+      <c r="D23" s="32">
+        <f>$B$5*$B$6*$B$7*$B$8*($B$9*Prices!D7+($B$10+$B$11)*Prices!E7)/1000000</f>
+        <v/>
+      </c>
+      <c r="E23" s="32">
+        <f>$B$5*$B$6*$B$7*$B$8*($B$9*Prices!D4+($B$10+$B$11)*Prices!E4)/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Agent-helper calls per month</t>
+        </is>
+      </c>
+      <c r="B24" s="15">
+        <f>$B$5*$B$6*$B$12</f>
+        <v/>
+      </c>
+      <c r="C24" s="15">
+        <f>$B$5*$B$6*$B$12</f>
+        <v/>
+      </c>
+      <c r="D24" s="15">
+        <f>$B$5*$B$6*$B$12</f>
+        <v/>
+      </c>
+      <c r="E24" s="15">
+        <f>$B$5*$B$6*$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Agent-helper cost</t>
+        </is>
+      </c>
+      <c r="B25" s="32">
+        <f>$B$5*$B$6*$B$12*($B$13*Prices!D6+($B$14+$B$15)*Prices!E6)/1000000</f>
+        <v/>
+      </c>
+      <c r="C25" s="32">
+        <f>$B$5*$B$6*$B$12*($B$13*Prices!D5+($B$14+$B$15)*Prices!E5)/1000000</f>
+        <v/>
+      </c>
+      <c r="D25" s="32">
+        <f>$B$5*$B$6*$B$12*($B$13*Prices!D7+($B$14+$B$15)*Prices!E7)/1000000</f>
+        <v/>
+      </c>
+      <c r="E25" s="32">
+        <f>$B$5*$B$6*$B$12*($B$13*Prices!D4+($B$14+$B$15)*Prices!E4)/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B26" s="32">
+        <f>B23+B25</f>
+        <v/>
+      </c>
+      <c r="C26" s="32">
+        <f>C23+C25</f>
+        <v/>
+      </c>
+      <c r="D26" s="32">
+        <f>D23+D25</f>
+        <v/>
+      </c>
+      <c r="E26" s="32">
+        <f>E23+E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B27" s="32">
+        <f>B26*$B$16</f>
+        <v/>
+      </c>
+      <c r="C27" s="32">
+        <f>C26*$B$16</f>
+        <v/>
+      </c>
+      <c r="D27" s="32">
+        <f>D26*$B$16</f>
+        <v/>
+      </c>
+      <c r="E27" s="32">
+        <f>E26*$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL per month (USD)</t>
+        </is>
+      </c>
+      <c r="B28" s="33">
+        <f>B26+B27</f>
+        <v/>
+      </c>
+      <c r="C28" s="33">
+        <f>C26+C27</f>
+        <v/>
+      </c>
+      <c r="D28" s="33">
+        <f>D26+D27</f>
+        <v/>
+      </c>
+      <c r="E28" s="33">
+        <f>E26+E27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL per month (SAR)</t>
+        </is>
+      </c>
+      <c r="B29" s="34">
+        <f>B28*$B$17</f>
+        <v/>
+      </c>
+      <c r="C29" s="34">
+        <f>C28*$B$17</f>
+        <v/>
+      </c>
+      <c r="D29" s="34">
+        <f>D28*$B$17</f>
+        <v/>
+      </c>
+      <c r="E29" s="34">
+        <f>E28*$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL per year (USD)</t>
+        </is>
+      </c>
+      <c r="B30" s="20">
+        <f>B28*12</f>
+        <v/>
+      </c>
+      <c r="C30" s="20">
+        <f>C28*12</f>
+        <v/>
+      </c>
+      <c r="D30" s="20">
+        <f>D28*12</f>
+        <v/>
+      </c>
+      <c r="E30" s="20">
+        <f>E28*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>TOTAL per year (SAR) - BUDGET LINE</t>
+        </is>
+      </c>
+      <c r="B31" s="35">
+        <f>B30*$B$17</f>
+        <v/>
+      </c>
+      <c r="C31" s="34">
+        <f>C30*$B$17</f>
+        <v/>
+      </c>
+      <c r="D31" s="34">
+        <f>D30*$B$17</f>
+        <v/>
+      </c>
+      <c r="E31" s="34">
+        <f>E30*$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>BUDGET LINE = Gemini 3.8 Flash at its standard 2027 price, the model the owner chose for auto-replies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Actual spend is recorded by the CRM itself: every AI call is logged with its tokens and cost (ai_calls). Replace the measured inputs above with the real monthly figures as auto-replies roll out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Billing: Google charges per token on a paid API key (no fixed fee). The free tier (~20 requests/day) cannot run production and lets Google use the data to improve its products; the paid tier does not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Not included: the engineering work to build auto-replies, and any WhatsApp/SMS sending fees.</t>
         </is>
       </c>
     </row>
@@ -683,7 +1085,192 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AI cost estimate - inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Blue cells are inputs: change them and every total recalculates. Yellow = the levers you will most likely change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Source / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Chats per month (today)</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Production 28 Sep - 7 Oct 2026: 298 chats in ~9 days = about 1,000/month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Growth multiplier</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Owner scenario: today x 5-6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>AI calls per chat (agent helper)</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Assumption: summaries, suggested replies, sentiment, enhance. Replace with the real figure from the ai_calls log after a few weeks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Input tokens per helper call</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Assumption: system prompt + chat history. Avg chat = 11 messages / ~630 characters (production).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Output tokens per helper call</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>300</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Customer messages per month (today)</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>5700</v>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Production: 1,717 customer messages in ~9 days = about 5,700/month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Input tokens per automated reply</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Assumption: full chat history + instructions + order context, sent on every customer message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Output tokens per automated reply</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Assumption: a short chat reply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>USD to SAR</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Fixed peg.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -749,10 +1336,10 @@
           <t>Current (free tier today)</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="36" t="n">
         <v>0.3</v>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="E4" s="36" t="n">
         <v>2.5</v>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -764,63 +1351,63 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna</t>
+          <t>Gemini 3.8 Flash (2026)</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Conversation - recommended</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E5" s="9" t="n">
-        <v>1.2</v>
+          <t>Auto-replies - recommended</t>
+        </is>
+      </c>
+      <c r="D5" s="36" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E5" s="36" t="n">
+        <v>3.75</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Budget tier of the GPT-5.6 family; enough for normal chat.</t>
+          <t>Introductory price until 31 Dec 2026. Output includes thinking tokens. Free tier ~20 requests/day - production needs a paid key.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>GPT-5 mini</t>
+          <t>Gemini 3.8 Flash (2027)</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Conversation</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E6" s="9" t="n">
-        <v>2</v>
+          <t>Auto-replies - BUDGET PRICE</t>
+        </is>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>7.5</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Same level, slightly stronger.</t>
+          <t>Standard price from 1 Jan 2027 - use this for the 2027 budget.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>GPT-5 nano</t>
+          <t>GPT-5.6 Luna</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -830,25 +1417,25 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Cheapest</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E7" s="9" t="n">
-        <v>0.4</v>
+          <t>Conversation (alternative)</t>
+        </is>
+      </c>
+      <c r="D7" s="36" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E7" s="36" t="n">
+        <v>1.2</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Weaker on Arabic and tricky cases.</t>
+          <t>Budget tier of the GPT-5.6 family; enough for normal chat.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.6 Terra</t>
+          <t>GPT-5 mini</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -858,58 +1445,114 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Mid / high (not needed)</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="n">
+          <t>Conversation</t>
+        </is>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="9" t="n">
-        <v>12</v>
-      </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>For comparison only.</t>
+          <t>Same level, slightly stronger.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>GPT-5 nano</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Cheapest</t>
+        </is>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E9" s="36" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Weaker on Arabic and tricky cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Terra</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Mid / high (not needed)</t>
+        </is>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>For comparison only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>GPT-5.6 Sol</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Top (not needed)</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D11" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E11" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>For comparison only.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Sources: morphllm.com/gemini-api-pricing; pricepertoken.com (gemini-2.5-flash); intuitionlabs.ai/articles/chatgpt-api-pricing-2026-token-costs-limits; morphllm.com/openai-api-pricing; layer3labs.io/guides/gpt-5-6-api-pricing. Prices change - re-check before deciding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Sources: morphllm.com/gemini-api-pricing; pricepertoken.com (gemini-2.5-flash); intuitionlabs.ai/articles/chatgpt-api-pricing-2026-token-costs-limits; morphllm.com/openai-api-pricing; layer3labs.io/guides/gpt-5-6-api-pricing; ai.google.dev/gemini-api/docs/pricing; layer3labs.io/guides/gemini-3-8-flash-pricing. Prices change - re-check before deciding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>OpenAI extras not applied: Batch API -50% (24h turnaround, not usable for live chat); cached input -50%.</t>
         </is>
@@ -920,13 +1563,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -953,274 +1596,342 @@
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Agent helper - today ($)</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>Agent helper - scaled ($)</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>AI answers customers - today ($)</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>AI answers customers - scaled ($)</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>Agent helper - scaled (SAR)</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>AI answers customers - scaled (SAR)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11">
+      <c r="A5" s="25">
         <f>Prices!A4</f>
         <v/>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="25">
         <f>Prices!C4</f>
         <v/>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="32">
         <f>Inputs!$B$5*Inputs!$B$7*(Inputs!$B$8*Prices!D4+Inputs!$B$9*Prices!E4)/1000000</f>
         <v/>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="32">
         <f>C5*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="32">
         <f>Inputs!$B$10*(Inputs!$B$11*Prices!D4+Inputs!$B$12*Prices!E4)/1000000</f>
         <v/>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="32">
         <f>E5*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="37">
         <f>D5*Inputs!$B$13</f>
         <v/>
       </c>
-      <c r="H5" s="13">
+      <c r="H5" s="37">
         <f>F5*Inputs!$B$13</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14">
+      <c r="A6" s="25">
         <f>Prices!A5</f>
         <v/>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="25">
         <f>Prices!C5</f>
         <v/>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="32">
         <f>Inputs!$B$5*Inputs!$B$7*(Inputs!$B$8*Prices!D5+Inputs!$B$9*Prices!E5)/1000000</f>
         <v/>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="32">
         <f>C6*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="32">
         <f>Inputs!$B$10*(Inputs!$B$11*Prices!D5+Inputs!$B$12*Prices!E5)/1000000</f>
         <v/>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="32">
         <f>E6*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="37">
         <f>D6*Inputs!$B$13</f>
         <v/>
       </c>
-      <c r="H6" s="16">
+      <c r="H6" s="37">
         <f>F6*Inputs!$B$13</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11">
+      <c r="A7" s="27">
         <f>Prices!A6</f>
         <v/>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="27">
         <f>Prices!C6</f>
         <v/>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="38">
         <f>Inputs!$B$5*Inputs!$B$7*(Inputs!$B$8*Prices!D6+Inputs!$B$9*Prices!E6)/1000000</f>
         <v/>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="38">
         <f>C7*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="38">
         <f>Inputs!$B$10*(Inputs!$B$11*Prices!D6+Inputs!$B$12*Prices!E6)/1000000</f>
         <v/>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="38">
         <f>E7*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="39">
         <f>D7*Inputs!$B$13</f>
         <v/>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="39">
         <f>F7*Inputs!$B$13</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11">
+      <c r="A8" s="25">
         <f>Prices!A7</f>
         <v/>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="25">
         <f>Prices!C7</f>
         <v/>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="32">
         <f>Inputs!$B$5*Inputs!$B$7*(Inputs!$B$8*Prices!D7+Inputs!$B$9*Prices!E7)/1000000</f>
         <v/>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="32">
         <f>C8*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="32">
         <f>Inputs!$B$10*(Inputs!$B$11*Prices!D7+Inputs!$B$12*Prices!E7)/1000000</f>
         <v/>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="32">
         <f>E8*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="37">
         <f>D8*Inputs!$B$13</f>
         <v/>
       </c>
-      <c r="H8" s="13">
+      <c r="H8" s="37">
         <f>F8*Inputs!$B$13</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11">
+      <c r="A9" s="25">
         <f>Prices!A8</f>
         <v/>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="25">
         <f>Prices!C8</f>
         <v/>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="32">
         <f>Inputs!$B$5*Inputs!$B$7*(Inputs!$B$8*Prices!D8+Inputs!$B$9*Prices!E8)/1000000</f>
         <v/>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="32">
         <f>C9*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="32">
         <f>Inputs!$B$10*(Inputs!$B$11*Prices!D8+Inputs!$B$12*Prices!E8)/1000000</f>
         <v/>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="32">
         <f>E9*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="37">
         <f>D9*Inputs!$B$13</f>
         <v/>
       </c>
-      <c r="H9" s="13">
+      <c r="H9" s="37">
         <f>F9*Inputs!$B$13</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11">
+      <c r="A10" s="25">
         <f>Prices!A9</f>
         <v/>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="25">
         <f>Prices!C9</f>
         <v/>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="32">
         <f>Inputs!$B$5*Inputs!$B$7*(Inputs!$B$8*Prices!D9+Inputs!$B$9*Prices!E9)/1000000</f>
         <v/>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="32">
         <f>C10*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="32">
         <f>Inputs!$B$10*(Inputs!$B$11*Prices!D9+Inputs!$B$12*Prices!E9)/1000000</f>
         <v/>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="32">
         <f>E10*Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="37">
         <f>D10*Inputs!$B$13</f>
         <v/>
       </c>
-      <c r="H10" s="13">
+      <c r="H10" s="37">
         <f>F10*Inputs!$B$13</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Agent helper = AI tools agents use today (summary, suggested reply, sentiment, enhance).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>AI answers customers = a future bot replying to every customer message, with the whole chat sent each time.</t>
-        </is>
+    <row r="11">
+      <c r="A11" s="25">
+        <f>Prices!A10</f>
+        <v/>
+      </c>
+      <c r="B11" s="25">
+        <f>Prices!C10</f>
+        <v/>
+      </c>
+      <c r="C11" s="32">
+        <f>Inputs!$B$5*Inputs!$B$7*(Inputs!$B$8*Prices!D10+Inputs!$B$9*Prices!E10)/1000000</f>
+        <v/>
+      </c>
+      <c r="D11" s="32">
+        <f>C11*Inputs!$B$6</f>
+        <v/>
+      </c>
+      <c r="E11" s="32">
+        <f>Inputs!$B$10*(Inputs!$B$11*Prices!D10+Inputs!$B$12*Prices!E10)/1000000</f>
+        <v/>
+      </c>
+      <c r="F11" s="32">
+        <f>E11*Inputs!$B$6</f>
+        <v/>
+      </c>
+      <c r="G11" s="37">
+        <f>D11*Inputs!$B$13</f>
+        <v/>
+      </c>
+      <c r="H11" s="37">
+        <f>F11*Inputs!$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25">
+        <f>Prices!A11</f>
+        <v/>
+      </c>
+      <c r="B12" s="25">
+        <f>Prices!C11</f>
+        <v/>
+      </c>
+      <c r="C12" s="32">
+        <f>Inputs!$B$5*Inputs!$B$7*(Inputs!$B$8*Prices!D11+Inputs!$B$9*Prices!E11)/1000000</f>
+        <v/>
+      </c>
+      <c r="D12" s="32">
+        <f>C12*Inputs!$B$6</f>
+        <v/>
+      </c>
+      <c r="E12" s="32">
+        <f>Inputs!$B$10*(Inputs!$B$11*Prices!D11+Inputs!$B$12*Prices!E11)/1000000</f>
+        <v/>
+      </c>
+      <c r="F12" s="32">
+        <f>E12*Inputs!$B$6</f>
+        <v/>
+      </c>
+      <c r="G12" s="37">
+        <f>D12*Inputs!$B$13</f>
+        <v/>
+      </c>
+      <c r="H12" s="37">
+        <f>F12*Inputs!$B$13</f>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Highlighted row = recommended for conversation. The Gemini row excludes "thinking" tokens (see Prices).</t>
+          <t>Agent helper = AI tools agents use today (summary, suggested reply, sentiment, enhance).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>AI answers customers = a future bot replying to every customer message, with the whole chat sent each time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Highlighted row = Gemini 3.8 Flash at its 2027 price (the budget price). These quick estimates exclude "thinking" tokens - the Budget 2027 sheet includes them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Replace the assumptions on Inputs with real numbers from the CRM's new ai_calls log once it has a few weeks of data.</t>
         </is>
@@ -1231,7 +1942,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1255,28 +1966,28 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="40" t="inlineStr">
         <is>
           <t>Agent replies (by a person): 1534</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="40" t="inlineStr">
         <is>
           <t>Automatic welcome messages: 78</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="40" t="inlineStr">
         <is>
           <t>Replies that were a quick reply: 426 (28%)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>Quick replies in the library (chat): 13; used at least once: 12</t>
         </is>
@@ -1317,252 +2028,252 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>رسالة ترحيب</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="41" t="n">
         <v>156</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="41" t="n">
         <v>156</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="42" t="inlineStr">
         <is>
           <t>السلام عليكم || !!!! || Where is my order ?!!!!!</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="41" t="inlineStr">
         <is>
           <t>رسالة انهاء المحادثة</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="41" t="n">
         <v>122</v>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="41" t="n">
         <v>120</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="41" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="42" t="inlineStr">
         <is>
           <t>هلا || شكرا || لم يرفق معها عصير</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>عدم الرد</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="41" t="n">
         <v>74</v>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="41" t="n">
         <v>40</v>
       </c>
-      <c r="D11" s="18" t="n">
+      <c r="D11" s="41" t="n">
         <v>34</v>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="42" t="inlineStr">
         <is>
           <t>Salam || هذي خدمة عملاء ... تحتاجون شكوى || تاخر تو وصل المندوب</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="41" t="inlineStr">
         <is>
           <t>تعويض عميل عنده حساب</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="41" t="n">
         <v>40</v>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="41" t="n">
         <v>37</v>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E12" s="42" t="inlineStr">
         <is>
           <t>Salam || Salam || Salam</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="41" t="inlineStr">
         <is>
           <t>الغاء</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="41" t="n">
         <v>23</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="41" t="n">
         <v>23</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="19" t="inlineStr">
+      <c r="E13" s="42" t="inlineStr">
         <is>
           <t>ابي الغيه طيب || غلط فيه || I ordered 2 pasta now, need with white sauce only not mix</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="41" t="inlineStr">
         <is>
           <t>استرداد مبلغ</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="19" t="inlineStr">
+      <c r="E14" s="42" t="inlineStr">
         <is>
           <t>Thanks || نعم صحيح || لا يعطيك العافيه</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="41" t="inlineStr">
         <is>
           <t>تعويض عميل ليس لديه حساب</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="41" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="18" t="n">
+      <c r="D15" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="19" t="inlineStr">
+      <c r="E15" s="42" t="inlineStr">
         <is>
           <t>Hello || تبشر بالجنة</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="41" t="inlineStr">
         <is>
           <t>Compensation customer with no account</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="18" t="n">
+      <c r="C16" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="19" t="inlineStr">
+      <c r="E16" s="42" t="inlineStr">
         <is>
           <t>Hello</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="41" t="inlineStr">
         <is>
           <t>متابعة</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n">
+      <c r="B17" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="18" t="n">
+      <c r="D17" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="19" t="inlineStr">
+      <c r="E17" s="42" t="inlineStr">
         <is>
           <t>مو اسلوب ذا طالع لي اقصى مده ساعه</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="41" t="inlineStr">
         <is>
           <t>Compensation for customer with account</t>
         </is>
       </c>
-      <c r="B18" s="18" t="n">
+      <c r="B18" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="18" t="n">
+      <c r="D18" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="19" t="inlineStr">
+      <c r="E18" s="42" t="inlineStr">
         <is>
           <t>Very bad service in the restaurant</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="41" t="inlineStr">
         <is>
           <t>تقديم</t>
         </is>
       </c>
-      <c r="B19" s="18" t="n">
+      <c r="B19" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="18" t="n">
+      <c r="C19" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D19" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="19" t="inlineStr">
+      <c r="E19" s="42" t="inlineStr">
         <is>
           <t>حابه اسأل عن التوظيف</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="41" t="inlineStr">
         <is>
           <t>Opening</t>
         </is>
       </c>
-      <c r="B20" s="18" t="n">
+      <c r="B20" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="18" t="n">
+      <c r="C20" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="19" t="inlineStr"/>
+      <c r="E20" s="42" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">

</xml_diff>